<commit_message>
Adding the Z-axis and intiating the full assembly
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78FE8A3-0B20-4815-926F-CA63BD90E003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6B5D46-3D34-4659-B06E-AA8CA40172C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8328" yWindow="624" windowWidth="9852" windowHeight="8256" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
   <sheets>
     <sheet name="DESIGN1_CAD_parameters(Sheet1)" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="25">
   <si>
     <t>Product_dia</t>
   </si>
@@ -102,6 +102,12 @@
   </si>
   <si>
     <t>VerticalStroke</t>
+  </si>
+  <si>
+    <t>BackArea</t>
+  </si>
+  <si>
+    <t>FrontArea</t>
   </si>
 </sst>
 </file>
@@ -970,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C3E246-7957-4EF1-A1E5-E58A01B1F4E8}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -1059,7 +1065,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -1093,7 +1099,7 @@
       </c>
       <c r="B11">
         <f>(4*B7)+(2*(B8+B9+B10))</f>
-        <v>412</v>
+        <v>452</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
@@ -1115,8 +1121,8 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <f>(2*B10)+(2*B8)+(8*B7)</f>
-        <v>624</v>
+        <f>(2*B10)+B23+B24+(8*B7)</f>
+        <v>764</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
@@ -1138,8 +1144,8 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <f>(5*B7)+(2*B8)+B9</f>
-        <v>395</v>
+        <f>(4*B7)+B23+B24+(2*B9)+(2*B10)</f>
+        <v>552</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -1151,7 +1157,7 @@
       </c>
       <c r="B16">
         <f>(4*B7)+(2*B8)+B9</f>
-        <v>332</v>
+        <v>372</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -1222,6 +1228,28 @@
         <v>85</v>
       </c>
       <c r="C22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23">
+        <v>150</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>50</v>
+      </c>
+      <c r="C24" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
A small change in the robot height
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6B5D46-3D34-4659-B06E-AA8CA40172C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C0D541-87F3-4D2A-8B55-4F319037483B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -1168,8 +1168,8 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <f>B20+B21+(B19/2)+50</f>
-        <v>168.5</v>
+        <f>B20+B21+(B19/2)</f>
+        <v>166.5</v>
       </c>
       <c r="C17" t="s">
         <v>1</v>
@@ -1191,7 +1191,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>127</v>
+        <v>223</v>
       </c>
       <c r="C19" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Some Updates on assemblies
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C0D541-87F3-4D2A-8B55-4F319037483B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039A99EA-62E7-40E5-AED0-D9D1B58A1803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="28">
   <si>
     <t>Product_dia</t>
   </si>
@@ -108,6 +108,15 @@
   </si>
   <si>
     <t>FrontArea</t>
+  </si>
+  <si>
+    <t>CylinderStroke</t>
+  </si>
+  <si>
+    <t>SideAreaWidth</t>
+  </si>
+  <si>
+    <t>BaseHeight</t>
   </si>
 </sst>
 </file>
@@ -976,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C3E246-7957-4EF1-A1E5-E58A01B1F4E8}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -1098,8 +1107,8 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <f>(4*B7)+(2*(B8+B9+B10))</f>
-        <v>452</v>
+        <f>(4*B7)+(2*(B8+B9+B10))+B26</f>
+        <v>652</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
@@ -1250,6 +1259,39 @@
         <v>50</v>
       </c>
       <c r="C24" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>75</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>200</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>70</v>
+      </c>
+      <c r="C27" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD boxes assemblies: base, power, pneumatic, and control
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039A99EA-62E7-40E5-AED0-D9D1B58A1803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0125596E-B98F-46FF-8999-D042FAB0F3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
   <si>
     <t>Product_dia</t>
   </si>
@@ -117,6 +117,33 @@
   </si>
   <si>
     <t>BaseHeight</t>
+  </si>
+  <si>
+    <t>BoxesClearance</t>
+  </si>
+  <si>
+    <t>BoxesWidth</t>
+  </si>
+  <si>
+    <t>PowerBoxLength</t>
+  </si>
+  <si>
+    <t>PneumaticBoxLength</t>
+  </si>
+  <si>
+    <t>ContolBoxLength</t>
+  </si>
+  <si>
+    <t>DistanceBetweenBoxes</t>
+  </si>
+  <si>
+    <t>BoxesHeight</t>
+  </si>
+  <si>
+    <t>ContolBoxWidth</t>
+  </si>
+  <si>
+    <t>ControlBoxHeight</t>
   </si>
 </sst>
 </file>
@@ -985,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C3E246-7957-4EF1-A1E5-E58A01B1F4E8}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -1119,7 +1146,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="C12" t="s">
         <v>1</v>
@@ -1130,8 +1157,8 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <f>(2*B10)+B23+B24+(8*B7)</f>
-        <v>764</v>
+        <f>(2*B10)+B23+B24+(4*B7)+B12</f>
+        <v>812</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
@@ -1292,6 +1319,106 @@
         <v>70</v>
       </c>
       <c r="C27" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>30</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <f>B26-(B28+B10)</f>
+        <v>140</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>300</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>200</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>160</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33">
+        <v>30</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34">
+        <v>170</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35">
+        <v>250</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36">
+        <v>120</v>
+      </c>
+      <c r="C36" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit Simulation CAD Files
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0125596E-B98F-46FF-8999-D042FAB0F3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD08C9B5-C552-4FA3-8A9B-0159BF2A854C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
+    <workbookView xWindow="8328" yWindow="624" windowWidth="9852" windowHeight="8256" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
   <sheets>
     <sheet name="DESIGN1_CAD_parameters(Sheet1)" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Adding Limit Switches for the Axises
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD08C9B5-C552-4FA3-8A9B-0159BF2A854C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B02EA78-8B59-4F73-A1A4-77BA7C47D870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8328" yWindow="624" windowWidth="9852" windowHeight="8256" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B13">
         <f>(2*B10)+B23+B24+(4*B7)+B12</f>
-        <v>812</v>
+        <v>912</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B15">
         <f>(4*B7)+B23+B24+(2*B9)+(2*B10)</f>
-        <v>552</v>
+        <v>652</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -1283,7 +1283,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Edits on Base Box
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B02EA78-8B59-4F73-A1A4-77BA7C47D870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4324BF-7CB3-4200-A297-09F60F55721B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8328" yWindow="624" windowWidth="9852" windowHeight="8256" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="38">
   <si>
     <t>Product_dia</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>ControlBoxHeight</t>
+  </si>
+  <si>
+    <t>BaseWoodThickness</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C3E246-7957-4EF1-A1E5-E58A01B1F4E8}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -1422,6 +1425,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37">
+        <v>7</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Mount The New Sorting Area
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C444BF2-00D5-4864-870A-51E557A672A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187529C9-9870-4261-876A-338B7B393047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8328" yWindow="624" windowWidth="9852" windowHeight="8256" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="B13">
         <f>(2*B10)+B23+B24+(4*B7)+B12</f>
-        <v>912</v>
+        <v>812</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B15">
         <f>(4*B7)+B23+B24+(2*B9)+(2*B10)</f>
-        <v>652</v>
+        <v>552</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -1284,7 +1284,7 @@
         <v>24</v>
       </c>
       <c r="B23">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Starting MatLab Multibody Simulation
</commit_message>
<xml_diff>
--- a/CAD/DESIGN1_CAD_parameters.xlsx
+++ b/CAD/DESIGN1_CAD_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Apps\AutodeskInventor\University\MCT333_Design_of_Mechatronics_Systems_1\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A2E7BA4-C49E-48A3-A208-F1745E04396F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67306A72-298E-465E-A301-5B5C3240CF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8328" yWindow="624" windowWidth="11664" windowHeight="11436" xr2:uid="{892A131F-3A33-47C6-BFB2-0EFCFF39DA2C}"/>
   </bookViews>
@@ -1216,8 +1216,8 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <f>B20+B21+(B19/2)</f>
-        <v>166.5</v>
+        <f>B20+B21+(B19/2)-30</f>
+        <v>136.5</v>
       </c>
       <c r="C17" t="s">
         <v>1</v>

</xml_diff>